<commit_message>
Ajustes en cargas de promociones
</commit_message>
<xml_diff>
--- a/application/views/template/sistema/archivos/excel/ventas_promociones_cargas/ventas_promociones_cargas.xlsx
+++ b/application/views/template/sistema/archivos/excel/ventas_promociones_cargas/ventas_promociones_cargas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\inetpub\wwwroot\strategix\php-7.4.27\clubdelpintoraxaltabrasil\application\views\template\sistema\archivos\excel\ventas_promociones_cargas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\inetpub\wwwroot\strategix\php_7.4.27\clubdelpintoraxaltabrasil\application\views\template\sistema\archivos\excel\ventas_promociones_cargas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEF78D1A-2328-472B-AF9D-D961AAF7DC43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE051DDD-5A51-4DBE-A49F-C7A3911F91C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{05105103-9B4C-4452-A2E6-A176226BDFDC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{05105103-9B4C-4452-A2E6-A176226BDFDC}"/>
   </bookViews>
   <sheets>
     <sheet name="productos" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -61,16 +61,29 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC82127"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -78,12 +91,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -118,6 +146,11 @@
       <tableStyleElement type="headerRow" dxfId="0"/>
     </tableStyle>
   </tableStyles>
+  <colors>
+    <mruColors>
+      <color rgb="FFC82127"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -426,7 +459,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B641ADA-4A97-49A6-8B49-4E0C8EB1CCE7}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="5.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
@@ -436,18 +469,276 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="2"/>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="2"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="2"/>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="2"/>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="2"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" s="2"/>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="2"/>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" s="2"/>
+      <c r="B30" s="2"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" s="2"/>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" s="2"/>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" s="2"/>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" s="2"/>
+      <c r="B34" s="2"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" s="2"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" s="2"/>
+      <c r="B36" s="2"/>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" s="2"/>
+      <c r="B37" s="2"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38" s="2"/>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39" s="2"/>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A40" s="2"/>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41" s="2"/>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A42" s="2"/>
+      <c r="B42" s="2"/>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A43" s="2"/>
+      <c r="B43" s="2"/>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A44" s="2"/>
+      <c r="B44" s="2"/>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>